<commit_message>
Rework CURRYiT budget split to follow deck revenue ramp, cleaner layout and reasons
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0189RpT3ueNgqmUTMfiRJ2Yn
</commit_message>
<xml_diff>
--- a/curryit-amazon-keywords/CURRYiT_Campaign_Structure_Media_Plan_Budget_Split.xlsx
+++ b/curryit-amazon-keywords/CURRYiT_Campaign_Structure_Media_Plan_Budget_Split.xlsx
@@ -33,7 +33,7 @@
     <numFmt numFmtId="167" formatCode="&quot;₹&quot;\ #,##0"/>
     <numFmt numFmtId="168" formatCode="₹#,##0"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -165,13 +165,24 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="15"/>
+    </font>
+    <font/>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
     </font>
     <font>
       <b val="1"/>
-      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -215,7 +226,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A9D08E"/>
+        <fgColor rgb="007B2C1E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8E5E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C0504D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -225,7 +261,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00F2DCDB"/>
       </patternFill>
     </fill>
   </fills>
@@ -360,23 +396,23 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00808080"/>
+        <color rgb="00A6A6A6"/>
       </left>
       <right style="thin">
-        <color rgb="00808080"/>
+        <color rgb="00A6A6A6"/>
       </right>
       <top style="thin">
-        <color rgb="00808080"/>
+        <color rgb="00A6A6A6"/>
       </top>
       <bottom style="thin">
-        <color rgb="00808080"/>
+        <color rgb="00A6A6A6"/>
       </bottom>
     </border>
     <border>
       <left/>
       <right/>
       <top style="thin">
-        <color rgb="00808080"/>
+        <color rgb="00A6A6A6"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -384,10 +420,10 @@
     <border>
       <left/>
       <right style="thin">
-        <color rgb="00808080"/>
+        <color rgb="00A6A6A6"/>
       </right>
       <top style="thin">
-        <color rgb="00808080"/>
+        <color rgb="00A6A6A6"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -396,23 +432,23 @@
       <left/>
       <right/>
       <top style="thin">
-        <color rgb="00808080"/>
+        <color rgb="00A6A6A6"/>
       </top>
       <bottom style="thin">
-        <color rgb="00808080"/>
+        <color rgb="00A6A6A6"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right style="thin">
-        <color rgb="00808080"/>
+        <color rgb="00A6A6A6"/>
       </right>
       <top style="thin">
-        <color rgb="00808080"/>
+        <color rgb="00A6A6A6"/>
       </top>
       <bottom style="thin">
-        <color rgb="00808080"/>
+        <color rgb="00A6A6A6"/>
       </bottom>
       <diagonal/>
     </border>
@@ -422,7 +458,7 @@
     <xf numFmtId="43" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="13" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -609,42 +645,93 @@
     <xf numFmtId="164" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="20" fillId="11" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="20" fillId="12" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="20" fillId="13" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="22" fillId="12" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="20" fillId="11" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="20" fillId="12" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="20" fillId="13" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="22" fillId="12" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="22" fillId="11" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="22" fillId="13" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="20" fillId="14" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="9" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="22" fillId="12" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="19" fillId="10" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="20" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="19" fillId="10" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="19" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -17981,7 +18068,7 @@
         <v>12</v>
       </c>
       <c r="H5" s="66" t="n">
-        <v>300000</v>
+        <v>200000</v>
       </c>
       <c r="I5" s="41">
         <f>H5/L5</f>
@@ -18087,7 +18174,7 @@
         <v>12</v>
       </c>
       <c r="H7" s="66" t="n">
-        <v>600000</v>
+        <v>450000</v>
       </c>
       <c r="I7" s="41">
         <f>H7/L7</f>
@@ -18193,7 +18280,7 @@
         <v>12</v>
       </c>
       <c r="H9" s="66" t="n">
-        <v>1000000</v>
+        <v>800000</v>
       </c>
       <c r="I9" s="41">
         <f>H9/L9</f>
@@ -18407,7 +18494,7 @@
       </c>
       <c r="C17" s="49" t="inlineStr">
         <is>
-          <t>Assumed the AOV as 1000 that is by taking the average of the 3 plant products pricing .</t>
+          <t>Assumed the AOV as ₹450 = CURRYiT combo pack of 3 pastes (given in the CURRYiT deck).</t>
         </is>
       </c>
       <c r="D17" s="61" t="n"/>
@@ -18442,1744 +18529,2074 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:K67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="58" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="68" t="inlineStr">
         <is>
-          <t>Budget Split – CURRYiT Chettinad (Month-wise, as per CURRYiT deck phases)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="69" t="inlineStr">
-        <is>
-          <t>A. Campaign type split (%)</t>
-        </is>
-      </c>
-      <c r="B3" s="70" t="n"/>
-      <c r="C3" s="70" t="n"/>
-      <c r="D3" s="70" t="n"/>
-      <c r="E3" s="70" t="n"/>
-      <c r="F3" s="70" t="n"/>
-      <c r="G3" s="70" t="n"/>
-      <c r="H3" s="70" t="n"/>
-      <c r="I3" s="70" t="n"/>
-      <c r="J3" s="71" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="72" t="inlineStr">
-        <is>
-          <t>Campaign type</t>
-        </is>
-      </c>
-      <c r="B4" s="72" t="inlineStr">
+          <t>CURRYiT Chettinad – Month-wise Budget Split (as per CURRYiT deck)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="69" t="inlineStr">
+        <is>
+          <t>Rule from deck: work backwards from the target → Revenue ÷ AOV ₹450 = orders ÷ CVR 8% = clicks × CPC ₹12 = spend. Spend only what each month's revenue target needs. Yellow = input, rest = formula.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="70" t="inlineStr">
+        <is>
+          <t>1. How much each month needs (from Media Planning sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="71" t="inlineStr"/>
+      <c r="B5" s="72" t="inlineStr">
         <is>
           <t>Month 1</t>
         </is>
       </c>
-      <c r="C4" s="72" t="inlineStr">
+      <c r="C5" s="72" t="inlineStr">
         <is>
           <t>Month 2</t>
         </is>
       </c>
-      <c r="D4" s="72" t="inlineStr">
+      <c r="D5" s="72" t="inlineStr">
         <is>
           <t>Month 3</t>
         </is>
       </c>
-      <c r="E4" s="72" t="inlineStr">
+      <c r="E5" s="72" t="inlineStr">
         <is>
           <t>Month 4</t>
         </is>
       </c>
-      <c r="F4" s="72" t="inlineStr">
+      <c r="F5" s="72" t="inlineStr">
         <is>
           <t>Month 5</t>
         </is>
       </c>
-      <c r="G4" s="72" t="inlineStr">
+      <c r="G5" s="72" t="inlineStr">
         <is>
           <t>Month 6</t>
         </is>
       </c>
-      <c r="H4" s="72" t="inlineStr">
-        <is>
-          <t>Phase logic</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="73" t="inlineStr">
-        <is>
-          <t>SP Keywords (Brand / Generic / Comp)</t>
-        </is>
-      </c>
-      <c r="B5" s="74" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="C5" s="74" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="D5" s="74" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="E5" s="74" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="F5" s="74" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="G5" s="74" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="H5" s="75" t="inlineStr">
-        <is>
-          <t>Biggest bucket all 6 months. Tightest targeting, best ROAS (deck).</t>
-        </is>
-      </c>
-      <c r="I5" s="70" t="n"/>
-      <c r="J5" s="71" t="n"/>
-    </row>
-    <row r="6" ht="32" customHeight="1">
-      <c r="A6" s="73" t="inlineStr">
-        <is>
-          <t>SP Auto</t>
-        </is>
-      </c>
-      <c r="B6" s="74" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C6" s="74" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D6" s="74" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E6" s="74" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F6" s="74" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="G6" s="74" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="H6" s="75" t="inlineStr">
-        <is>
-          <t>High in M1–2 to find keywords; cut later as winners move to Exact.</t>
-        </is>
-      </c>
-      <c r="I6" s="70" t="n"/>
-      <c r="J6" s="71" t="n"/>
-    </row>
-    <row r="7" ht="32" customHeight="1">
-      <c r="A7" s="73" t="inlineStr">
-        <is>
-          <t>SP Product Targeting (CT + IP)</t>
-        </is>
-      </c>
-      <c r="B7" s="74" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C7" s="74" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D7" s="74" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="E7" s="74" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="F7" s="74" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="G7" s="74" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="H7" s="75" t="inlineStr">
-        <is>
-          <t>Show ad on competitor pages from day 1 (deck).</t>
-        </is>
-      </c>
-      <c r="I7" s="70" t="n"/>
-      <c r="J7" s="71" t="n"/>
-    </row>
-    <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="73" t="inlineStr">
-        <is>
-          <t>SB Video</t>
-        </is>
-      </c>
-      <c r="B8" s="74" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="C8" s="74" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="D8" s="74" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="E8" s="74" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="F8" s="74" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="G8" s="74" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="H8" s="75" t="inlineStr">
-        <is>
-          <t>15-min cooking video = best format for food (deck). Flat all months.</t>
-        </is>
-      </c>
-      <c r="I8" s="70" t="n"/>
-      <c r="J8" s="71" t="n"/>
-    </row>
-    <row r="9" ht="32" customHeight="1">
-      <c r="A9" s="73" t="inlineStr">
-        <is>
-          <t>SB Brand (combo) – new</t>
-        </is>
-      </c>
-      <c r="B9" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="74" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E9" s="74" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F9" s="74" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="G9" s="74" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="H9" s="75" t="inlineStr">
-        <is>
-          <t>Deck rule: start in Month 3, sells the combo not the single pouch.</t>
-        </is>
-      </c>
-      <c r="I9" s="70" t="n"/>
-      <c r="J9" s="71" t="n"/>
-    </row>
-    <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="73" t="inlineStr">
-        <is>
-          <t>SD (Retargeting + Audiences)</t>
-        </is>
-      </c>
-      <c r="B10" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="74" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="E10" s="74" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="F10" s="74" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="G10" s="74" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="H10" s="75" t="inlineStr">
-        <is>
-          <t>Deck puts "retarget people who viewed" in M3–4. Viewer pool from M1–2 ads is ready by then.</t>
-        </is>
-      </c>
-      <c r="I10" s="70" t="n"/>
-      <c r="J10" s="71" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="76" t="inlineStr">
-        <is>
-          <t>Total (must be 100%)</t>
-        </is>
-      </c>
-      <c r="B11" s="77">
-        <f>SUM(B5:B10)</f>
-        <v/>
-      </c>
-      <c r="C11" s="77">
-        <f>SUM(C5:C10)</f>
-        <v/>
-      </c>
-      <c r="D11" s="77">
-        <f>SUM(D5:D10)</f>
-        <v/>
-      </c>
-      <c r="E11" s="77">
-        <f>SUM(E5:E10)</f>
-        <v/>
-      </c>
-      <c r="F11" s="77">
-        <f>SUM(F5:F10)</f>
-        <v/>
-      </c>
-      <c r="G11" s="77">
-        <f>SUM(G5:G10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="69" t="inlineStr">
-        <is>
-          <t>B. Campaign-wise budget (₹ per month) – total spend taken from your Media Planning sheet</t>
-        </is>
-      </c>
-      <c r="B14" s="70" t="n"/>
-      <c r="C14" s="70" t="n"/>
-      <c r="D14" s="70" t="n"/>
-      <c r="E14" s="70" t="n"/>
-      <c r="F14" s="70" t="n"/>
-      <c r="G14" s="70" t="n"/>
-      <c r="H14" s="70" t="n"/>
-      <c r="I14" s="70" t="n"/>
-      <c r="J14" s="71" t="n"/>
+      <c r="H5" s="72" t="inlineStr">
+        <is>
+          <t>6-month total</t>
+        </is>
+      </c>
+      <c r="I5" s="73" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="74" t="inlineStr">
+        <is>
+          <t>Deck phase</t>
+        </is>
+      </c>
+      <c r="B6" s="75" t="inlineStr">
+        <is>
+          <t>Get started</t>
+        </is>
+      </c>
+      <c r="C6" s="75" t="inlineStr">
+        <is>
+          <t>Get started</t>
+        </is>
+      </c>
+      <c r="D6" s="76" t="inlineStr">
+        <is>
+          <t>Grow</t>
+        </is>
+      </c>
+      <c r="E6" s="76" t="inlineStr">
+        <is>
+          <t>Grow</t>
+        </is>
+      </c>
+      <c r="F6" s="77" t="inlineStr">
+        <is>
+          <t>Hit target</t>
+        </is>
+      </c>
+      <c r="G6" s="77" t="inlineStr">
+        <is>
+          <t>Hit target</t>
+        </is>
+      </c>
+      <c r="H6" s="78" t="inlineStr"/>
+      <c r="I6" s="79" t="inlineStr">
+        <is>
+          <t>Deck: "Split your budget across six months"</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="74" t="inlineStr">
+        <is>
+          <t>Revenue target</t>
+        </is>
+      </c>
+      <c r="B7" s="80">
+        <f>'Media Planning'!H5</f>
+        <v/>
+      </c>
+      <c r="C7" s="80">
+        <f>'Media Planning'!H6</f>
+        <v/>
+      </c>
+      <c r="D7" s="81">
+        <f>'Media Planning'!H7</f>
+        <v/>
+      </c>
+      <c r="E7" s="81">
+        <f>'Media Planning'!H8</f>
+        <v/>
+      </c>
+      <c r="F7" s="82">
+        <f>'Media Planning'!H9</f>
+        <v/>
+      </c>
+      <c r="G7" s="82">
+        <f>'Media Planning'!H10</f>
+        <v/>
+      </c>
+      <c r="H7" s="83">
+        <f>SUM(B7:G7)</f>
+        <v/>
+      </c>
+      <c r="I7" s="79" t="inlineStr">
+        <is>
+          <t>Deck: ₹1.4L→₹3L (M1–2), ₹3L→₹6L (M3–4), ₹6L→₹10L (M5–6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="74" t="inlineStr">
+        <is>
+          <t>Orders needed</t>
+        </is>
+      </c>
+      <c r="B8" s="84">
+        <f>'Media Planning'!I5</f>
+        <v/>
+      </c>
+      <c r="C8" s="84">
+        <f>'Media Planning'!I6</f>
+        <v/>
+      </c>
+      <c r="D8" s="85">
+        <f>'Media Planning'!I7</f>
+        <v/>
+      </c>
+      <c r="E8" s="85">
+        <f>'Media Planning'!I8</f>
+        <v/>
+      </c>
+      <c r="F8" s="86">
+        <f>'Media Planning'!I9</f>
+        <v/>
+      </c>
+      <c r="G8" s="86">
+        <f>'Media Planning'!I10</f>
+        <v/>
+      </c>
+      <c r="H8" s="87">
+        <f>SUM(B8:G8)</f>
+        <v/>
+      </c>
+      <c r="I8" s="79" t="inlineStr">
+        <is>
+          <t>Revenue ÷ AOV ₹450</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="74" t="inlineStr">
+        <is>
+          <t>Clicks needed</t>
+        </is>
+      </c>
+      <c r="B9" s="84">
+        <f>'Media Planning'!F5</f>
+        <v/>
+      </c>
+      <c r="C9" s="84">
+        <f>'Media Planning'!F6</f>
+        <v/>
+      </c>
+      <c r="D9" s="85">
+        <f>'Media Planning'!F7</f>
+        <v/>
+      </c>
+      <c r="E9" s="85">
+        <f>'Media Planning'!F8</f>
+        <v/>
+      </c>
+      <c r="F9" s="86">
+        <f>'Media Planning'!F9</f>
+        <v/>
+      </c>
+      <c r="G9" s="86">
+        <f>'Media Planning'!F10</f>
+        <v/>
+      </c>
+      <c r="H9" s="87">
+        <f>SUM(B9:G9)</f>
+        <v/>
+      </c>
+      <c r="I9" s="79" t="inlineStr">
+        <is>
+          <t>Spend ÷ CPC ₹12</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="74" t="inlineStr">
+        <is>
+          <t>Ad spend needed</t>
+        </is>
+      </c>
+      <c r="B10" s="88">
+        <f>'Media Planning'!B5</f>
+        <v/>
+      </c>
+      <c r="C10" s="88">
+        <f>'Media Planning'!B6</f>
+        <v/>
+      </c>
+      <c r="D10" s="83">
+        <f>'Media Planning'!B7</f>
+        <v/>
+      </c>
+      <c r="E10" s="83">
+        <f>'Media Planning'!B8</f>
+        <v/>
+      </c>
+      <c r="F10" s="89">
+        <f>'Media Planning'!B9</f>
+        <v/>
+      </c>
+      <c r="G10" s="89">
+        <f>'Media Planning'!B10</f>
+        <v/>
+      </c>
+      <c r="H10" s="83">
+        <f>SUM(B10:G10)</f>
+        <v/>
+      </c>
+      <c r="I10" s="79" t="inlineStr">
+        <is>
+          <t>Revenue ÷ ROAS 3 (deck: ₹10L ÷ ₹3,33,300 = 3.0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="90" t="inlineStr">
+        <is>
+          <t>What the deck asks each phase →  M1–2: fix listing, early reviews, fix shipping, find best SKU.   M3–4: spend more on what works, start brand campaigns, push combo, retarget viewers.   M5–6: ranking improves, repeat buyers, Subscribe &amp; Save, tighten – do not expand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="70" t="inlineStr">
+        <is>
+          <t>2. Split by the 6 campaign types in the deck (%)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="72" t="inlineStr">
         <is>
-          <t>Campaign Name</t>
+          <t>Campaign type (deck)</t>
         </is>
       </c>
       <c r="B15" s="72" t="inlineStr">
         <is>
-          <t>Share in type</t>
+          <t>Month 1</t>
         </is>
       </c>
       <c r="C15" s="72" t="inlineStr">
         <is>
+          <t>Month 2</t>
+        </is>
+      </c>
+      <c r="D15" s="72" t="inlineStr">
+        <is>
+          <t>Month 3</t>
+        </is>
+      </c>
+      <c r="E15" s="72" t="inlineStr">
+        <is>
+          <t>Month 4</t>
+        </is>
+      </c>
+      <c r="F15" s="72" t="inlineStr">
+        <is>
+          <t>Month 5</t>
+        </is>
+      </c>
+      <c r="G15" s="72" t="inlineStr">
+        <is>
+          <t>Month 6</t>
+        </is>
+      </c>
+      <c r="H15" s="72" t="inlineStr">
+        <is>
+          <t>6-mo ₹</t>
+        </is>
+      </c>
+      <c r="I15" s="73" t="inlineStr">
+        <is>
+          <t>Why (valid reason)</t>
+        </is>
+      </c>
+      <c r="J15" s="91" t="n"/>
+      <c r="K15" s="92" t="n"/>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="74" t="inlineStr">
+        <is>
+          <t>SP Exact (keywords)</t>
+        </is>
+      </c>
+      <c r="B16" s="93" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="C16" s="93" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="D16" s="93" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="E16" s="93" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F16" s="93" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="G16" s="93" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H16" s="83">
+        <f>B10*B16+C10*C16+D10*D16+E10*E16+F10*F16+G10*G16</f>
+        <v/>
+      </c>
+      <c r="I16" s="79" t="inlineStr">
+        <is>
+          <t>Deck: "tightest targeting, best ROAS". Biggest share every month; falls a little as SB/SD come in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="74" t="inlineStr">
+        <is>
+          <t>SP Auto</t>
+        </is>
+      </c>
+      <c r="B17" s="93" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C17" s="93" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D17" s="93" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E17" s="93" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F17" s="93" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G17" s="93" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H17" s="83">
+        <f>B10*B17+C10*C17+D10*D17+E10*E17+F10*F17+G10*G17</f>
+        <v/>
+      </c>
+      <c r="I17" s="79" t="inlineStr">
+        <is>
+          <t>Deck: "for finding new keywords". Needed most in M1–2 to find what converts; cut once winners move to Exact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="74" t="inlineStr">
+        <is>
+          <t>SP Product Targeting</t>
+        </is>
+      </c>
+      <c r="B18" s="93" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C18" s="93" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D18" s="93" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E18" s="93" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F18" s="93" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G18" s="93" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="H18" s="83">
+        <f>B10*B18+C10*C18+D10*D18+E10*E18+F10*F18+G10*G18</f>
+        <v/>
+      </c>
+      <c r="I18" s="79" t="inlineStr">
+        <is>
+          <t>Deck: "show your ad on competitor pages". Strong at start to take shoppers already on Chettinad/paste pages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="74" t="inlineStr">
+        <is>
+          <t>SB Video</t>
+        </is>
+      </c>
+      <c r="B19" s="93" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C19" s="93" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D19" s="93" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E19" s="93" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F19" s="93" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G19" s="93" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H19" s="83">
+        <f>B10*B19+C10*C19+D10*D19+E10*E19+F10*F19+G10*G19</f>
+        <v/>
+      </c>
+      <c r="I19" s="79" t="inlineStr">
+        <is>
+          <t>Deck: "15-min cooking video, best format for food". Kept flat so CURRYiT is always on top of search.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="74" t="inlineStr">
+        <is>
+          <t>SB Brand (combo)</t>
+        </is>
+      </c>
+      <c r="B20" s="93" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="93" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="93" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E20" s="93" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F20" s="93" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G20" s="93" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H20" s="83">
+        <f>B10*B20+C10*C20+D10*D20+E10*E20+F10*F20+G10*G20</f>
+        <v/>
+      </c>
+      <c r="I20" s="79" t="inlineStr">
+        <is>
+          <t>Deck: "Start in Month 3. Sells the combo". 0 before M3; grows in M5–6 because combo = AOV ₹450.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="74" t="inlineStr">
+        <is>
+          <t>SD Retargeting</t>
+        </is>
+      </c>
+      <c r="B21" s="93" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="93" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="93" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E21" s="93" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F21" s="93" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G21" s="93" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="H21" s="83">
+        <f>B10*B21+C10*C21+D10*D21+E10*E21+F10*F21+G10*G21</f>
+        <v/>
+      </c>
+      <c r="I21" s="79" t="inlineStr">
+        <is>
+          <t>Deck puts "retarget people who viewed" in M3–4. M1–2 ads build the viewer pool first; M5–6 adds repeat buyers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="94" t="inlineStr">
+        <is>
+          <t>Check (must be 100%)</t>
+        </is>
+      </c>
+      <c r="B22" s="95">
+        <f>SUM(B16:B21)</f>
+        <v/>
+      </c>
+      <c r="C22" s="95">
+        <f>SUM(C16:C21)</f>
+        <v/>
+      </c>
+      <c r="D22" s="95">
+        <f>SUM(D16:D21)</f>
+        <v/>
+      </c>
+      <c r="E22" s="95">
+        <f>SUM(E16:E21)</f>
+        <v/>
+      </c>
+      <c r="F22" s="95">
+        <f>SUM(F16:F21)</f>
+        <v/>
+      </c>
+      <c r="G22" s="95">
+        <f>SUM(G16:G21)</f>
+        <v/>
+      </c>
+      <c r="H22" s="83">
+        <f>SUM(H16:H21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="70" t="inlineStr">
+        <is>
+          <t>3. Campaign-wise budget (₹ per month) – your campaigns from SP / SB / SD sheets</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="72" t="inlineStr">
+        <is>
+          <t>Campaign name</t>
+        </is>
+      </c>
+      <c r="B25" s="72" t="inlineStr">
+        <is>
+          <t>Share</t>
+        </is>
+      </c>
+      <c r="C25" s="72" t="inlineStr">
+        <is>
           <t>Month 1</t>
         </is>
       </c>
-      <c r="D15" s="72" t="inlineStr">
+      <c r="D25" s="72" t="inlineStr">
         <is>
           <t>Month 2</t>
         </is>
       </c>
-      <c r="E15" s="72" t="inlineStr">
+      <c r="E25" s="72" t="inlineStr">
         <is>
           <t>Month 3</t>
         </is>
       </c>
-      <c r="F15" s="72" t="inlineStr">
+      <c r="F25" s="72" t="inlineStr">
         <is>
           <t>Month 4</t>
         </is>
       </c>
-      <c r="G15" s="72" t="inlineStr">
+      <c r="G25" s="72" t="inlineStr">
         <is>
           <t>Month 5</t>
         </is>
       </c>
-      <c r="H15" s="72" t="inlineStr">
+      <c r="H25" s="72" t="inlineStr">
         <is>
           <t>Month 6</t>
         </is>
       </c>
-      <c r="I15" s="72" t="inlineStr">
-        <is>
-          <t>6-month total</t>
-        </is>
-      </c>
-      <c r="J15" s="72" t="inlineStr">
+      <c r="I25" s="72" t="inlineStr">
+        <is>
+          <t>6-mo total</t>
+        </is>
+      </c>
+      <c r="J25" s="72" t="inlineStr">
+        <is>
+          <t>Exp. orders (6 mo)</t>
+        </is>
+      </c>
+      <c r="K25" s="73" t="inlineStr">
         <is>
           <t>Why this share</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="76" t="inlineStr">
-        <is>
-          <t>Total monthly spend (Media Planning)</t>
-        </is>
-      </c>
-      <c r="B16" s="78" t="inlineStr"/>
-      <c r="C16" s="79">
-        <f>'Media Planning'!B5</f>
-        <v/>
-      </c>
-      <c r="D16" s="79">
-        <f>'Media Planning'!B6</f>
-        <v/>
-      </c>
-      <c r="E16" s="79">
-        <f>'Media Planning'!B7</f>
-        <v/>
-      </c>
-      <c r="F16" s="79">
-        <f>'Media Planning'!B8</f>
-        <v/>
-      </c>
-      <c r="G16" s="79">
-        <f>'Media Planning'!B9</f>
-        <v/>
-      </c>
-      <c r="H16" s="79">
-        <f>'Media Planning'!B10</f>
-        <v/>
-      </c>
-      <c r="I16" s="79">
-        <f>SUM(C16:H16)</f>
-        <v/>
-      </c>
-      <c r="J16" s="78" t="inlineStr"/>
-    </row>
-    <row r="17" ht="44" customHeight="1">
-      <c r="A17" s="75" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="96" t="inlineStr">
+        <is>
+          <t>SP Exact (keywords)   (gets 45/45/35/35/32/32% of monthly spend, M1→M6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="44" customHeight="1">
+      <c r="A27" s="79" t="inlineStr">
+        <is>
+          <t>SP/ChettinadChicken/Generic KWs/Exact</t>
+        </is>
+      </c>
+      <c r="B27" s="93" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C27" s="80">
+        <f>B$10*B$16*0.3</f>
+        <v/>
+      </c>
+      <c r="D27" s="80">
+        <f>C$10*C$16*0.3</f>
+        <v/>
+      </c>
+      <c r="E27" s="81">
+        <f>D$10*D$16*0.3</f>
+        <v/>
+      </c>
+      <c r="F27" s="81">
+        <f>E$10*E$16*0.3</f>
+        <v/>
+      </c>
+      <c r="G27" s="82">
+        <f>F$10*F$16*0.3</f>
+        <v/>
+      </c>
+      <c r="H27" s="82">
+        <f>G$10*G$16*0.3</f>
+        <v/>
+      </c>
+      <c r="I27" s="83">
+        <f>SUM(C27:H27)</f>
+        <v/>
+      </c>
+      <c r="J27" s="97">
+        <f>ROUND(I27/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K27" s="79" t="inlineStr">
+        <is>
+          <t>Generic = 4,190 searches/mo (Chettinad 1,980 + chicken curry masala 1,490 + paste/RTC 720) – biggest relevant pool. Deck: product keywords = Priority 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="79" t="inlineStr">
+        <is>
+          <t>SP/ChettinadChicken/Generic KWs/Phrase</t>
+        </is>
+      </c>
+      <c r="B28" s="93" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C28" s="80">
+        <f>B$10*B$16*0.2</f>
+        <v/>
+      </c>
+      <c r="D28" s="80">
+        <f>C$10*C$16*0.2</f>
+        <v/>
+      </c>
+      <c r="E28" s="81">
+        <f>D$10*D$16*0.2</f>
+        <v/>
+      </c>
+      <c r="F28" s="81">
+        <f>E$10*E$16*0.2</f>
+        <v/>
+      </c>
+      <c r="G28" s="82">
+        <f>F$10*F$16*0.2</f>
+        <v/>
+      </c>
+      <c r="H28" s="82">
+        <f>G$10*G$16*0.2</f>
+        <v/>
+      </c>
+      <c r="I28" s="83">
+        <f>SUM(C28:H28)</f>
+        <v/>
+      </c>
+      <c r="J28" s="97">
+        <f>ROUND(I28/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K28" s="79" t="inlineStr">
+        <is>
+          <t>Same keywords, catches longer searches like "chettinad masala for chicken".</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="79" t="inlineStr">
+        <is>
+          <t>SP/ChettinadChicken/Generic KWs/Broad</t>
+        </is>
+      </c>
+      <c r="B29" s="93" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C29" s="80">
+        <f>B$10*B$16*0.1</f>
+        <v/>
+      </c>
+      <c r="D29" s="80">
+        <f>C$10*C$16*0.1</f>
+        <v/>
+      </c>
+      <c r="E29" s="81">
+        <f>D$10*D$16*0.1</f>
+        <v/>
+      </c>
+      <c r="F29" s="81">
+        <f>E$10*E$16*0.1</f>
+        <v/>
+      </c>
+      <c r="G29" s="82">
+        <f>F$10*F$16*0.1</f>
+        <v/>
+      </c>
+      <c r="H29" s="82">
+        <f>G$10*G$16*0.1</f>
+        <v/>
+      </c>
+      <c r="I29" s="83">
+        <f>SUM(C29:H29)</f>
+        <v/>
+      </c>
+      <c r="J29" s="97">
+        <f>ROUND(I29/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K29" s="79" t="inlineStr">
+        <is>
+          <t>Only for discovery; negated vs Phrase so no overlap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="79" t="inlineStr">
+        <is>
+          <t>SP/ChettinadChicken/Comp KWs/Exact</t>
+        </is>
+      </c>
+      <c r="B30" s="93" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="C30" s="80">
+        <f>B$10*B$16*0.12</f>
+        <v/>
+      </c>
+      <c r="D30" s="80">
+        <f>C$10*C$16*0.12</f>
+        <v/>
+      </c>
+      <c r="E30" s="81">
+        <f>D$10*D$16*0.12</f>
+        <v/>
+      </c>
+      <c r="F30" s="81">
+        <f>E$10*E$16*0.12</f>
+        <v/>
+      </c>
+      <c r="G30" s="82">
+        <f>F$10*F$16*0.12</f>
+        <v/>
+      </c>
+      <c r="H30" s="82">
+        <f>G$10*G$16*0.12</f>
+        <v/>
+      </c>
+      <c r="I30" s="83">
+        <f>SUM(C30:H30)</f>
+        <v/>
+      </c>
+      <c r="J30" s="97">
+        <f>ROUND(I30/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K30" s="79" t="inlineStr">
+        <is>
+          <t>Comp searches only 820/mo and need switching; kept lower than Generic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="79" t="inlineStr">
+        <is>
+          <t>SP/ChettinadChicken/Comp KWs/Phrase</t>
+        </is>
+      </c>
+      <c r="B31" s="93" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="C31" s="80">
+        <f>B$10*B$16*0.08</f>
+        <v/>
+      </c>
+      <c r="D31" s="80">
+        <f>C$10*C$16*0.08</f>
+        <v/>
+      </c>
+      <c r="E31" s="81">
+        <f>D$10*D$16*0.08</f>
+        <v/>
+      </c>
+      <c r="F31" s="81">
+        <f>E$10*E$16*0.08</f>
+        <v/>
+      </c>
+      <c r="G31" s="82">
+        <f>F$10*F$16*0.08</f>
+        <v/>
+      </c>
+      <c r="H31" s="82">
+        <f>G$10*G$16*0.08</f>
+        <v/>
+      </c>
+      <c r="I31" s="83">
+        <f>SUM(C31:H31)</f>
+        <v/>
+      </c>
+      <c r="J31" s="97">
+        <f>ROUND(I31/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K31" s="79" t="inlineStr"/>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="79" t="inlineStr">
+        <is>
+          <t>SP/ChettinadChicken/Comp KWs/Broad</t>
+        </is>
+      </c>
+      <c r="B32" s="93" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C32" s="80">
+        <f>B$10*B$16*0.05</f>
+        <v/>
+      </c>
+      <c r="D32" s="80">
+        <f>C$10*C$16*0.05</f>
+        <v/>
+      </c>
+      <c r="E32" s="81">
+        <f>D$10*D$16*0.05</f>
+        <v/>
+      </c>
+      <c r="F32" s="81">
+        <f>E$10*E$16*0.05</f>
+        <v/>
+      </c>
+      <c r="G32" s="82">
+        <f>F$10*F$16*0.05</f>
+        <v/>
+      </c>
+      <c r="H32" s="82">
+        <f>G$10*G$16*0.05</f>
+        <v/>
+      </c>
+      <c r="I32" s="83">
+        <f>SUM(C32:H32)</f>
+        <v/>
+      </c>
+      <c r="J32" s="97">
+        <f>ROUND(I32/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K32" s="79" t="inlineStr"/>
+    </row>
+    <row r="33" ht="44" customHeight="1">
+      <c r="A33" s="79" t="inlineStr">
         <is>
           <t>SP/ChettinadChicken/Brand KWs/Exact</t>
         </is>
       </c>
-      <c r="B17" s="74" t="n">
+      <c r="B33" s="93" t="n">
         <v>0.08</v>
       </c>
-      <c r="C17" s="80">
-        <f>C$16*B$5*0.08</f>
-        <v/>
-      </c>
-      <c r="D17" s="80">
-        <f>D$16*C$5*0.08</f>
-        <v/>
-      </c>
-      <c r="E17" s="80">
-        <f>E$16*D$5*0.08</f>
-        <v/>
-      </c>
-      <c r="F17" s="80">
-        <f>F$16*E$5*0.08</f>
-        <v/>
-      </c>
-      <c r="G17" s="80">
-        <f>G$16*F$5*0.08</f>
-        <v/>
-      </c>
-      <c r="H17" s="80">
-        <f>H$16*G$5*0.08</f>
-        <v/>
-      </c>
-      <c r="I17" s="81">
-        <f>SUM(C17:H17)</f>
-        <v/>
-      </c>
-      <c r="J17" s="75" t="inlineStr">
-        <is>
-          <t>Brand search: curry it 2,400 + curryit 1,300 = 3,700/mo. Cheap; protect own name.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="75" t="inlineStr">
+      <c r="C33" s="80">
+        <f>B$10*B$16*0.08</f>
+        <v/>
+      </c>
+      <c r="D33" s="80">
+        <f>C$10*C$16*0.08</f>
+        <v/>
+      </c>
+      <c r="E33" s="81">
+        <f>D$10*D$16*0.08</f>
+        <v/>
+      </c>
+      <c r="F33" s="81">
+        <f>E$10*E$16*0.08</f>
+        <v/>
+      </c>
+      <c r="G33" s="82">
+        <f>F$10*F$16*0.08</f>
+        <v/>
+      </c>
+      <c r="H33" s="82">
+        <f>G$10*G$16*0.08</f>
+        <v/>
+      </c>
+      <c r="I33" s="83">
+        <f>SUM(C33:H33)</f>
+        <v/>
+      </c>
+      <c r="J33" s="97">
+        <f>ROUND(I33/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K33" s="79" t="inlineStr">
+        <is>
+          <t>Brand searches 3,700/mo (curry it 2,400 + curryit 1,300). Shopper already wants CURRYiT, so cheap clicks; just protect the top slot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="79" t="inlineStr">
         <is>
           <t>SP/ChettinadChicken/Brand KWs/Phrase</t>
         </is>
       </c>
-      <c r="B18" s="74" t="n">
+      <c r="B34" s="93" t="n">
         <v>0.05</v>
       </c>
-      <c r="C18" s="80">
-        <f>C$16*B$5*0.05</f>
-        <v/>
-      </c>
-      <c r="D18" s="80">
-        <f>D$16*C$5*0.05</f>
-        <v/>
-      </c>
-      <c r="E18" s="80">
-        <f>E$16*D$5*0.05</f>
-        <v/>
-      </c>
-      <c r="F18" s="80">
-        <f>F$16*E$5*0.05</f>
-        <v/>
-      </c>
-      <c r="G18" s="80">
-        <f>G$16*F$5*0.05</f>
-        <v/>
-      </c>
-      <c r="H18" s="80">
-        <f>H$16*G$5*0.05</f>
-        <v/>
-      </c>
-      <c r="I18" s="81">
-        <f>SUM(C18:H18)</f>
-        <v/>
-      </c>
-      <c r="J18" s="75" t="inlineStr">
-        <is>
-          <t>Catches "curryit chettinad…" variations.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="75" t="inlineStr">
+      <c r="C34" s="80">
+        <f>B$10*B$16*0.05</f>
+        <v/>
+      </c>
+      <c r="D34" s="80">
+        <f>C$10*C$16*0.05</f>
+        <v/>
+      </c>
+      <c r="E34" s="81">
+        <f>D$10*D$16*0.05</f>
+        <v/>
+      </c>
+      <c r="F34" s="81">
+        <f>E$10*E$16*0.05</f>
+        <v/>
+      </c>
+      <c r="G34" s="82">
+        <f>F$10*F$16*0.05</f>
+        <v/>
+      </c>
+      <c r="H34" s="82">
+        <f>G$10*G$16*0.05</f>
+        <v/>
+      </c>
+      <c r="I34" s="83">
+        <f>SUM(C34:H34)</f>
+        <v/>
+      </c>
+      <c r="J34" s="97">
+        <f>ROUND(I34/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K34" s="79" t="inlineStr"/>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="79" t="inlineStr">
         <is>
           <t>SP/ChettinadChicken/Brand KWs/Broad</t>
         </is>
       </c>
-      <c r="B19" s="74" t="n">
+      <c r="B35" s="93" t="n">
         <v>0.02</v>
       </c>
-      <c r="C19" s="80">
-        <f>C$16*B$5*0.02</f>
-        <v/>
-      </c>
-      <c r="D19" s="80">
-        <f>D$16*C$5*0.02</f>
-        <v/>
-      </c>
-      <c r="E19" s="80">
-        <f>E$16*D$5*0.02</f>
-        <v/>
-      </c>
-      <c r="F19" s="80">
-        <f>F$16*E$5*0.02</f>
-        <v/>
-      </c>
-      <c r="G19" s="80">
-        <f>G$16*F$5*0.02</f>
-        <v/>
-      </c>
-      <c r="H19" s="80">
-        <f>H$16*G$5*0.02</f>
-        <v/>
-      </c>
-      <c r="I19" s="81">
-        <f>SUM(C19:H19)</f>
-        <v/>
-      </c>
-      <c r="J19" s="75" t="inlineStr">
-        <is>
-          <t>Small – only to find new brand terms.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="44" customHeight="1">
-      <c r="A20" s="75" t="inlineStr">
-        <is>
-          <t>SP/ChettinadChicken/Generic KWs/Exact</t>
-        </is>
-      </c>
-      <c r="B20" s="74" t="n">
+      <c r="C35" s="80">
+        <f>B$10*B$16*0.02</f>
+        <v/>
+      </c>
+      <c r="D35" s="80">
+        <f>C$10*C$16*0.02</f>
+        <v/>
+      </c>
+      <c r="E35" s="81">
+        <f>D$10*D$16*0.02</f>
+        <v/>
+      </c>
+      <c r="F35" s="81">
+        <f>E$10*E$16*0.02</f>
+        <v/>
+      </c>
+      <c r="G35" s="82">
+        <f>F$10*F$16*0.02</f>
+        <v/>
+      </c>
+      <c r="H35" s="82">
+        <f>G$10*G$16*0.02</f>
+        <v/>
+      </c>
+      <c r="I35" s="83">
+        <f>SUM(C35:H35)</f>
+        <v/>
+      </c>
+      <c r="J35" s="97">
+        <f>ROUND(I35/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K35" s="79" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="96" t="inlineStr">
+        <is>
+          <t>SP Auto   (gets 20/20/10/10/8/8% of monthly spend, M1→M6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="79" t="inlineStr">
+        <is>
+          <t>SP/ChettinadChicken/Auto</t>
+        </is>
+      </c>
+      <c r="B37" s="93" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" s="80">
+        <f>B$10*B$17*1.0</f>
+        <v/>
+      </c>
+      <c r="D37" s="80">
+        <f>C$10*C$17*1.0</f>
+        <v/>
+      </c>
+      <c r="E37" s="81">
+        <f>D$10*D$17*1.0</f>
+        <v/>
+      </c>
+      <c r="F37" s="81">
+        <f>E$10*E$17*1.0</f>
+        <v/>
+      </c>
+      <c r="G37" s="82">
+        <f>F$10*F$17*1.0</f>
+        <v/>
+      </c>
+      <c r="H37" s="82">
+        <f>G$10*G$17*1.0</f>
+        <v/>
+      </c>
+      <c r="I37" s="83">
+        <f>SUM(C37:H37)</f>
+        <v/>
+      </c>
+      <c r="J37" s="97">
+        <f>ROUND(I37/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K37" s="79" t="inlineStr">
+        <is>
+          <t>Only Auto campaign. Weekly search-term check (deck).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="96" t="inlineStr">
+        <is>
+          <t>SP Product Targeting   (gets 20/20/15/15/12/12% of monthly spend, M1→M6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="79" t="inlineStr">
+        <is>
+          <t>SP/IP/CompTar – competitor ASINs</t>
+        </is>
+      </c>
+      <c r="B39" s="93" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="C39" s="80">
+        <f>B$10*B$18*0.55</f>
+        <v/>
+      </c>
+      <c r="D39" s="80">
+        <f>C$10*C$18*0.55</f>
+        <v/>
+      </c>
+      <c r="E39" s="81">
+        <f>D$10*D$18*0.55</f>
+        <v/>
+      </c>
+      <c r="F39" s="81">
+        <f>E$10*E$18*0.55</f>
+        <v/>
+      </c>
+      <c r="G39" s="82">
+        <f>F$10*F$18*0.55</f>
+        <v/>
+      </c>
+      <c r="H39" s="82">
+        <f>G$10*G$18*0.55</f>
+        <v/>
+      </c>
+      <c r="I39" s="83">
+        <f>SUM(C39:H39)</f>
+        <v/>
+      </c>
+      <c r="J39" s="97">
+        <f>ROUND(I39/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K39" s="79" t="inlineStr">
+        <is>
+          <t>Competitor pages = shoppers ready to buy a Chettinad/curry product today.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="79" t="inlineStr">
+        <is>
+          <t>SP/CT – category</t>
+        </is>
+      </c>
+      <c r="B40" s="93" t="n">
         <v>0.3</v>
       </c>
-      <c r="C20" s="80">
-        <f>C$16*B$5*0.3</f>
-        <v/>
-      </c>
-      <c r="D20" s="80">
-        <f>D$16*C$5*0.3</f>
-        <v/>
-      </c>
-      <c r="E20" s="80">
-        <f>E$16*D$5*0.3</f>
-        <v/>
-      </c>
-      <c r="F20" s="80">
-        <f>F$16*E$5*0.3</f>
-        <v/>
-      </c>
-      <c r="G20" s="80">
-        <f>G$16*F$5*0.3</f>
-        <v/>
-      </c>
-      <c r="H20" s="80">
-        <f>H$16*G$5*0.3</f>
-        <v/>
-      </c>
-      <c r="I20" s="81">
-        <f>SUM(C20:H20)</f>
-        <v/>
-      </c>
-      <c r="J20" s="75" t="inlineStr">
-        <is>
-          <t>Main money bucket: Chettinad 1,980 + chicken curry masala 1,490 + paste/RTC 720 = 4,190 searches/mo. Deck: product keywords = Priority 1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="75" t="inlineStr">
-        <is>
-          <t>SP/ChettinadChicken/Generic KWs/Phrase</t>
-        </is>
-      </c>
-      <c r="B21" s="74" t="n">
+      <c r="C40" s="80">
+        <f>B$10*B$18*0.3</f>
+        <v/>
+      </c>
+      <c r="D40" s="80">
+        <f>C$10*C$18*0.3</f>
+        <v/>
+      </c>
+      <c r="E40" s="81">
+        <f>D$10*D$18*0.3</f>
+        <v/>
+      </c>
+      <c r="F40" s="81">
+        <f>E$10*E$18*0.3</f>
+        <v/>
+      </c>
+      <c r="G40" s="82">
+        <f>F$10*F$18*0.3</f>
+        <v/>
+      </c>
+      <c r="H40" s="82">
+        <f>G$10*G$18*0.3</f>
+        <v/>
+      </c>
+      <c r="I40" s="83">
+        <f>SUM(C40:H40)</f>
+        <v/>
+      </c>
+      <c r="J40" s="97">
+        <f>ROUND(I40/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K40" s="79" t="inlineStr">
+        <is>
+          <t>Wider reach, lower bid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="79" t="inlineStr">
+        <is>
+          <t>SP/IP/BrandTar – own ASINs</t>
+        </is>
+      </c>
+      <c r="B41" s="93" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C41" s="80">
+        <f>B$10*B$18*0.15</f>
+        <v/>
+      </c>
+      <c r="D41" s="80">
+        <f>C$10*C$18*0.15</f>
+        <v/>
+      </c>
+      <c r="E41" s="81">
+        <f>D$10*D$18*0.15</f>
+        <v/>
+      </c>
+      <c r="F41" s="81">
+        <f>E$10*E$18*0.15</f>
+        <v/>
+      </c>
+      <c r="G41" s="82">
+        <f>F$10*F$18*0.15</f>
+        <v/>
+      </c>
+      <c r="H41" s="82">
+        <f>G$10*G$18*0.15</f>
+        <v/>
+      </c>
+      <c r="I41" s="83">
+        <f>SUM(C41:H41)</f>
+        <v/>
+      </c>
+      <c r="J41" s="97">
+        <f>ROUND(I41/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K41" s="79" t="inlineStr">
+        <is>
+          <t>Stops competitors taking our own page; cross-sells other CURRYiT pastes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="96" t="inlineStr">
+        <is>
+          <t>SB Video   (gets 15/15/15/15/15/15% of monthly spend, M1→M6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="44" customHeight="1">
+      <c r="A43" s="79" t="inlineStr">
+        <is>
+          <t>SB/Video/Generic Chettinad kws-Exact</t>
+        </is>
+      </c>
+      <c r="B43" s="93" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C43" s="80">
+        <f>B$10*B$19*0.3</f>
+        <v/>
+      </c>
+      <c r="D43" s="80">
+        <f>C$10*C$19*0.3</f>
+        <v/>
+      </c>
+      <c r="E43" s="81">
+        <f>D$10*D$19*0.3</f>
+        <v/>
+      </c>
+      <c r="F43" s="81">
+        <f>E$10*E$19*0.3</f>
+        <v/>
+      </c>
+      <c r="G43" s="82">
+        <f>F$10*F$19*0.3</f>
+        <v/>
+      </c>
+      <c r="H43" s="82">
+        <f>G$10*G$19*0.3</f>
+        <v/>
+      </c>
+      <c r="I43" s="83">
+        <f>SUM(C43:H43)</f>
+        <v/>
+      </c>
+      <c r="J43" s="97">
+        <f>ROUND(I43/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K43" s="79" t="inlineStr">
+        <is>
+          <t>New customers come from generic search; video shows "15 mins, 3 steps, no grinding".</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="79" t="inlineStr">
+        <is>
+          <t>SB/Video/Generic Chettinad kws-Phrase</t>
+        </is>
+      </c>
+      <c r="B44" s="93" t="n">
         <v>0.2</v>
       </c>
-      <c r="C21" s="80">
-        <f>C$16*B$5*0.2</f>
-        <v/>
-      </c>
-      <c r="D21" s="80">
-        <f>D$16*C$5*0.2</f>
-        <v/>
-      </c>
-      <c r="E21" s="80">
-        <f>E$16*D$5*0.2</f>
-        <v/>
-      </c>
-      <c r="F21" s="80">
-        <f>F$16*E$5*0.2</f>
-        <v/>
-      </c>
-      <c r="G21" s="80">
-        <f>G$16*F$5*0.2</f>
-        <v/>
-      </c>
-      <c r="H21" s="80">
-        <f>H$16*G$5*0.2</f>
-        <v/>
-      </c>
-      <c r="I21" s="81">
-        <f>SUM(C21:H21)</f>
-        <v/>
-      </c>
-      <c r="J21" s="75" t="inlineStr">
-        <is>
-          <t>Same keywords, more search variations.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="75" t="inlineStr">
-        <is>
-          <t>SP/ChettinadChicken/Generic KWs/Broad</t>
-        </is>
-      </c>
-      <c r="B22" s="74" t="n">
+      <c r="C44" s="80">
+        <f>B$10*B$19*0.2</f>
+        <v/>
+      </c>
+      <c r="D44" s="80">
+        <f>C$10*C$19*0.2</f>
+        <v/>
+      </c>
+      <c r="E44" s="81">
+        <f>D$10*D$19*0.2</f>
+        <v/>
+      </c>
+      <c r="F44" s="81">
+        <f>E$10*E$19*0.2</f>
+        <v/>
+      </c>
+      <c r="G44" s="82">
+        <f>F$10*F$19*0.2</f>
+        <v/>
+      </c>
+      <c r="H44" s="82">
+        <f>G$10*G$19*0.2</f>
+        <v/>
+      </c>
+      <c r="I44" s="83">
+        <f>SUM(C44:H44)</f>
+        <v/>
+      </c>
+      <c r="J44" s="97">
+        <f>ROUND(I44/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K44" s="79" t="inlineStr"/>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="79" t="inlineStr">
+        <is>
+          <t>SB/Video/Brand kws-Exact</t>
+        </is>
+      </c>
+      <c r="B45" s="93" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C45" s="80">
+        <f>B$10*B$19*0.15</f>
+        <v/>
+      </c>
+      <c r="D45" s="80">
+        <f>C$10*C$19*0.15</f>
+        <v/>
+      </c>
+      <c r="E45" s="81">
+        <f>D$10*D$19*0.15</f>
+        <v/>
+      </c>
+      <c r="F45" s="81">
+        <f>E$10*E$19*0.15</f>
+        <v/>
+      </c>
+      <c r="G45" s="82">
+        <f>F$10*F$19*0.15</f>
+        <v/>
+      </c>
+      <c r="H45" s="82">
+        <f>G$10*G$19*0.15</f>
+        <v/>
+      </c>
+      <c r="I45" s="83">
+        <f>SUM(C45:H45)</f>
+        <v/>
+      </c>
+      <c r="J45" s="97">
+        <f>ROUND(I45/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K45" s="79" t="inlineStr">
+        <is>
+          <t>Brand video converts searchers who are comparing CURRYiT variants.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="79" t="inlineStr">
+        <is>
+          <t>SB/Video/Brand kws-Phrase</t>
+        </is>
+      </c>
+      <c r="B46" s="93" t="n">
         <v>0.1</v>
       </c>
-      <c r="C22" s="80">
-        <f>C$16*B$5*0.1</f>
-        <v/>
-      </c>
-      <c r="D22" s="80">
-        <f>D$16*C$5*0.1</f>
-        <v/>
-      </c>
-      <c r="E22" s="80">
-        <f>E$16*D$5*0.1</f>
-        <v/>
-      </c>
-      <c r="F22" s="80">
-        <f>F$16*E$5*0.1</f>
-        <v/>
-      </c>
-      <c r="G22" s="80">
-        <f>G$16*F$5*0.1</f>
-        <v/>
-      </c>
-      <c r="H22" s="80">
-        <f>H$16*G$5*0.1</f>
-        <v/>
-      </c>
-      <c r="I22" s="81">
-        <f>SUM(C22:H22)</f>
-        <v/>
-      </c>
-      <c r="J22" s="75" t="inlineStr">
-        <is>
-          <t>Discovery only; negated vs Phrase.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="44" customHeight="1">
-      <c r="A23" s="75" t="inlineStr">
-        <is>
-          <t>SP/ChettinadChicken/Comp KWs/Exact</t>
-        </is>
-      </c>
-      <c r="B23" s="74" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="C23" s="80">
-        <f>C$16*B$5*0.12</f>
-        <v/>
-      </c>
-      <c r="D23" s="80">
-        <f>D$16*C$5*0.12</f>
-        <v/>
-      </c>
-      <c r="E23" s="80">
-        <f>E$16*D$5*0.12</f>
-        <v/>
-      </c>
-      <c r="F23" s="80">
-        <f>F$16*E$5*0.12</f>
-        <v/>
-      </c>
-      <c r="G23" s="80">
-        <f>G$16*F$5*0.12</f>
-        <v/>
-      </c>
-      <c r="H23" s="80">
-        <f>H$16*G$5*0.12</f>
-        <v/>
-      </c>
-      <c r="I23" s="81">
-        <f>SUM(C23:H23)</f>
-        <v/>
-      </c>
-      <c r="J23" s="75" t="inlineStr">
-        <is>
-          <t>Comp keyword volume is small (Chettinad comp 230 + chicken masala brands 520 + paste brands 70 = 820/mo), and their buyers convert lower.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="75" t="inlineStr">
-        <is>
-          <t>SP/ChettinadChicken/Comp KWs/Phrase</t>
-        </is>
-      </c>
-      <c r="B24" s="74" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="C24" s="80">
-        <f>C$16*B$5*0.08</f>
-        <v/>
-      </c>
-      <c r="D24" s="80">
-        <f>D$16*C$5*0.08</f>
-        <v/>
-      </c>
-      <c r="E24" s="80">
-        <f>E$16*D$5*0.08</f>
-        <v/>
-      </c>
-      <c r="F24" s="80">
-        <f>F$16*E$5*0.08</f>
-        <v/>
-      </c>
-      <c r="G24" s="80">
-        <f>G$16*F$5*0.08</f>
-        <v/>
-      </c>
-      <c r="H24" s="80">
-        <f>H$16*G$5*0.08</f>
-        <v/>
-      </c>
-      <c r="I24" s="81">
-        <f>SUM(C24:H24)</f>
-        <v/>
-      </c>
-      <c r="J24" s="75" t="inlineStr">
-        <is>
-          <t>Same as above.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="75" t="inlineStr">
-        <is>
-          <t>SP/ChettinadChicken/Comp KWs/Broad</t>
-        </is>
-      </c>
-      <c r="B25" s="74" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="C25" s="80">
-        <f>C$16*B$5*0.05</f>
-        <v/>
-      </c>
-      <c r="D25" s="80">
-        <f>D$16*C$5*0.05</f>
-        <v/>
-      </c>
-      <c r="E25" s="80">
-        <f>E$16*D$5*0.05</f>
-        <v/>
-      </c>
-      <c r="F25" s="80">
-        <f>F$16*E$5*0.05</f>
-        <v/>
-      </c>
-      <c r="G25" s="80">
-        <f>G$16*F$5*0.05</f>
-        <v/>
-      </c>
-      <c r="H25" s="80">
-        <f>H$16*G$5*0.05</f>
-        <v/>
-      </c>
-      <c r="I25" s="81">
-        <f>SUM(C25:H25)</f>
-        <v/>
-      </c>
-      <c r="J25" s="75" t="inlineStr">
-        <is>
-          <t>Small test.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="75" t="inlineStr">
-        <is>
-          <t>SP/ChettinadChicken/Auto</t>
-        </is>
-      </c>
-      <c r="B26" s="74" t="n">
+      <c r="C46" s="80">
+        <f>B$10*B$19*0.1</f>
+        <v/>
+      </c>
+      <c r="D46" s="80">
+        <f>C$10*C$19*0.1</f>
+        <v/>
+      </c>
+      <c r="E46" s="81">
+        <f>D$10*D$19*0.1</f>
+        <v/>
+      </c>
+      <c r="F46" s="81">
+        <f>E$10*E$19*0.1</f>
+        <v/>
+      </c>
+      <c r="G46" s="82">
+        <f>F$10*F$19*0.1</f>
+        <v/>
+      </c>
+      <c r="H46" s="82">
+        <f>G$10*G$19*0.1</f>
+        <v/>
+      </c>
+      <c r="I46" s="83">
+        <f>SUM(C46:H46)</f>
+        <v/>
+      </c>
+      <c r="J46" s="97">
+        <f>ROUND(I46/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K46" s="79" t="inlineStr"/>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="79" t="inlineStr">
+        <is>
+          <t>SB/Video/Comp kws-Exact</t>
+        </is>
+      </c>
+      <c r="B47" s="93" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C47" s="80">
+        <f>B$10*B$19*0.15</f>
+        <v/>
+      </c>
+      <c r="D47" s="80">
+        <f>C$10*C$19*0.15</f>
+        <v/>
+      </c>
+      <c r="E47" s="81">
+        <f>D$10*D$19*0.15</f>
+        <v/>
+      </c>
+      <c r="F47" s="81">
+        <f>E$10*E$19*0.15</f>
+        <v/>
+      </c>
+      <c r="G47" s="82">
+        <f>F$10*F$19*0.15</f>
+        <v/>
+      </c>
+      <c r="H47" s="82">
+        <f>G$10*G$19*0.15</f>
+        <v/>
+      </c>
+      <c r="I47" s="83">
+        <f>SUM(C47:H47)</f>
+        <v/>
+      </c>
+      <c r="J47" s="97">
+        <f>ROUND(I47/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K47" s="79" t="inlineStr">
+        <is>
+          <t>Video is the best way to make a competitor shopper stop and switch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="79" t="inlineStr">
+        <is>
+          <t>SB/Video/Comp kws-Phrase</t>
+        </is>
+      </c>
+      <c r="B48" s="93" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C48" s="80">
+        <f>B$10*B$19*0.1</f>
+        <v/>
+      </c>
+      <c r="D48" s="80">
+        <f>C$10*C$19*0.1</f>
+        <v/>
+      </c>
+      <c r="E48" s="81">
+        <f>D$10*D$19*0.1</f>
+        <v/>
+      </c>
+      <c r="F48" s="81">
+        <f>E$10*E$19*0.1</f>
+        <v/>
+      </c>
+      <c r="G48" s="82">
+        <f>F$10*F$19*0.1</f>
+        <v/>
+      </c>
+      <c r="H48" s="82">
+        <f>G$10*G$19*0.1</f>
+        <v/>
+      </c>
+      <c r="I48" s="83">
+        <f>SUM(C48:H48)</f>
+        <v/>
+      </c>
+      <c r="J48" s="97">
+        <f>ROUND(I48/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K48" s="79" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="96" t="inlineStr">
+        <is>
+          <t>SB Brand (combo)   (gets 0/0/10/10/15/15% of monthly spend, M1→M6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="79" t="inlineStr">
+        <is>
+          <t>SB Brand – Product Collection (Combo-3) – ADD from M3</t>
+        </is>
+      </c>
+      <c r="B50" s="93" t="n">
         <v>1</v>
       </c>
-      <c r="C26" s="80">
-        <f>C$16*B$6*1.0</f>
-        <v/>
-      </c>
-      <c r="D26" s="80">
-        <f>D$16*C$6*1.0</f>
-        <v/>
-      </c>
-      <c r="E26" s="80">
-        <f>E$16*D$6*1.0</f>
-        <v/>
-      </c>
-      <c r="F26" s="80">
-        <f>F$16*E$6*1.0</f>
-        <v/>
-      </c>
-      <c r="G26" s="80">
-        <f>G$16*F$6*1.0</f>
-        <v/>
-      </c>
-      <c r="H26" s="80">
-        <f>H$16*G$6*1.0</f>
-        <v/>
-      </c>
-      <c r="I26" s="81">
-        <f>SUM(C26:H26)</f>
-        <v/>
-      </c>
-      <c r="J26" s="75" t="inlineStr">
-        <is>
-          <t>Only Auto campaign. Check search term report weekly (deck).</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="44" customHeight="1">
-      <c r="A27" s="75" t="inlineStr">
-        <is>
-          <t>SP/IP/CompTar (competitor ASINs)</t>
-        </is>
-      </c>
-      <c r="B27" s="74" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="C27" s="80">
-        <f>C$16*B$7*0.55</f>
-        <v/>
-      </c>
-      <c r="D27" s="80">
-        <f>D$16*C$7*0.55</f>
-        <v/>
-      </c>
-      <c r="E27" s="80">
-        <f>E$16*D$7*0.55</f>
-        <v/>
-      </c>
-      <c r="F27" s="80">
-        <f>F$16*E$7*0.55</f>
-        <v/>
-      </c>
-      <c r="G27" s="80">
-        <f>G$16*F$7*0.55</f>
-        <v/>
-      </c>
-      <c r="H27" s="80">
-        <f>H$16*G$7*0.55</f>
-        <v/>
-      </c>
-      <c r="I27" s="81">
-        <f>SUM(C27:H27)</f>
-        <v/>
-      </c>
-      <c r="J27" s="75" t="inlineStr">
-        <is>
-          <t>Show CURRYiT on competitor product pages (deck). Pitch: paste, ghee, no preservatives.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="75" t="inlineStr">
-        <is>
-          <t>SP/CT (category)</t>
-        </is>
-      </c>
-      <c r="B28" s="74" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C28" s="80">
-        <f>C$16*B$7*0.3</f>
-        <v/>
-      </c>
-      <c r="D28" s="80">
-        <f>D$16*C$7*0.3</f>
-        <v/>
-      </c>
-      <c r="E28" s="80">
-        <f>E$16*D$7*0.3</f>
-        <v/>
-      </c>
-      <c r="F28" s="80">
-        <f>F$16*E$7*0.3</f>
-        <v/>
-      </c>
-      <c r="G28" s="80">
-        <f>G$16*F$7*0.3</f>
-        <v/>
-      </c>
-      <c r="H28" s="80">
-        <f>H$16*G$7*0.3</f>
-        <v/>
-      </c>
-      <c r="I28" s="81">
-        <f>SUM(C28:H28)</f>
-        <v/>
-      </c>
-      <c r="J28" s="75" t="inlineStr">
-        <is>
-          <t>Wider category reach at lower bid.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="75" t="inlineStr">
-        <is>
-          <t>SP/IP/BrandTar (own ASINs)</t>
-        </is>
-      </c>
-      <c r="B29" s="74" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="C29" s="80">
-        <f>C$16*B$7*0.15</f>
-        <v/>
-      </c>
-      <c r="D29" s="80">
-        <f>D$16*C$7*0.15</f>
-        <v/>
-      </c>
-      <c r="E29" s="80">
-        <f>E$16*D$7*0.15</f>
-        <v/>
-      </c>
-      <c r="F29" s="80">
-        <f>F$16*E$7*0.15</f>
-        <v/>
-      </c>
-      <c r="G29" s="80">
-        <f>G$16*F$7*0.15</f>
-        <v/>
-      </c>
-      <c r="H29" s="80">
-        <f>H$16*G$7*0.15</f>
-        <v/>
-      </c>
-      <c r="I29" s="81">
-        <f>SUM(C29:H29)</f>
-        <v/>
-      </c>
-      <c r="J29" s="75" t="inlineStr">
-        <is>
-          <t>Defend own pages, cross-sell other CURRYiT pastes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="75" t="inlineStr">
-        <is>
-          <t>SB/Video/Brand kws-Exact</t>
-        </is>
-      </c>
-      <c r="B30" s="74" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="C30" s="80">
-        <f>C$16*B$8*0.15</f>
-        <v/>
-      </c>
-      <c r="D30" s="80">
-        <f>D$16*C$8*0.15</f>
-        <v/>
-      </c>
-      <c r="E30" s="80">
-        <f>E$16*D$8*0.15</f>
-        <v/>
-      </c>
-      <c r="F30" s="80">
-        <f>F$16*E$8*0.15</f>
-        <v/>
-      </c>
-      <c r="G30" s="80">
-        <f>G$16*F$8*0.15</f>
-        <v/>
-      </c>
-      <c r="H30" s="80">
-        <f>H$16*G$8*0.15</f>
-        <v/>
-      </c>
-      <c r="I30" s="81">
-        <f>SUM(C30:H30)</f>
-        <v/>
-      </c>
-      <c r="J30" s="75" t="inlineStr">
-        <is>
-          <t>Brand video for people already searching CURRYiT.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="75" t="inlineStr">
-        <is>
-          <t>SB/Video/Brand kws-Phrase</t>
-        </is>
-      </c>
-      <c r="B31" s="74" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C31" s="80">
-        <f>C$16*B$8*0.1</f>
-        <v/>
-      </c>
-      <c r="D31" s="80">
-        <f>D$16*C$8*0.1</f>
-        <v/>
-      </c>
-      <c r="E31" s="80">
-        <f>E$16*D$8*0.1</f>
-        <v/>
-      </c>
-      <c r="F31" s="80">
-        <f>F$16*E$8*0.1</f>
-        <v/>
-      </c>
-      <c r="G31" s="80">
-        <f>G$16*F$8*0.1</f>
-        <v/>
-      </c>
-      <c r="H31" s="80">
-        <f>H$16*G$8*0.1</f>
-        <v/>
-      </c>
-      <c r="I31" s="81">
-        <f>SUM(C31:H31)</f>
-        <v/>
-      </c>
-      <c r="J31" s="75" t="inlineStr"/>
-    </row>
-    <row r="32" ht="44" customHeight="1">
-      <c r="A32" s="75" t="inlineStr">
-        <is>
-          <t>SB/Video/Generic Chettinad kws-Exact</t>
-        </is>
-      </c>
-      <c r="B32" s="74" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C32" s="80">
-        <f>C$16*B$8*0.3</f>
-        <v/>
-      </c>
-      <c r="D32" s="80">
-        <f>D$16*C$8*0.3</f>
-        <v/>
-      </c>
-      <c r="E32" s="80">
-        <f>E$16*D$8*0.3</f>
-        <v/>
-      </c>
-      <c r="F32" s="80">
-        <f>F$16*E$8*0.3</f>
-        <v/>
-      </c>
-      <c r="G32" s="80">
-        <f>G$16*F$8*0.3</f>
-        <v/>
-      </c>
-      <c r="H32" s="80">
-        <f>H$16*G$8*0.3</f>
-        <v/>
-      </c>
-      <c r="I32" s="81">
-        <f>SUM(C32:H32)</f>
-        <v/>
-      </c>
-      <c r="J32" s="75" t="inlineStr">
-        <is>
-          <t>Most new customers come from generic searches; video shows "15 mins, 3 steps".</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="75" t="inlineStr">
-        <is>
-          <t>SB/Video/Generic Chettinad kws-Phrase</t>
-        </is>
-      </c>
-      <c r="B33" s="74" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C33" s="80">
-        <f>C$16*B$8*0.2</f>
-        <v/>
-      </c>
-      <c r="D33" s="80">
-        <f>D$16*C$8*0.2</f>
-        <v/>
-      </c>
-      <c r="E33" s="80">
-        <f>E$16*D$8*0.2</f>
-        <v/>
-      </c>
-      <c r="F33" s="80">
-        <f>F$16*E$8*0.2</f>
-        <v/>
-      </c>
-      <c r="G33" s="80">
-        <f>G$16*F$8*0.2</f>
-        <v/>
-      </c>
-      <c r="H33" s="80">
-        <f>H$16*G$8*0.2</f>
-        <v/>
-      </c>
-      <c r="I33" s="81">
-        <f>SUM(C33:H33)</f>
-        <v/>
-      </c>
-      <c r="J33" s="75" t="inlineStr"/>
-    </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="75" t="inlineStr">
-        <is>
-          <t>SB/Video/Comp kws-Exact</t>
-        </is>
-      </c>
-      <c r="B34" s="74" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="C34" s="80">
-        <f>C$16*B$8*0.15</f>
-        <v/>
-      </c>
-      <c r="D34" s="80">
-        <f>D$16*C$8*0.15</f>
-        <v/>
-      </c>
-      <c r="E34" s="80">
-        <f>E$16*D$8*0.15</f>
-        <v/>
-      </c>
-      <c r="F34" s="80">
-        <f>F$16*E$8*0.15</f>
-        <v/>
-      </c>
-      <c r="G34" s="80">
-        <f>G$16*F$8*0.15</f>
-        <v/>
-      </c>
-      <c r="H34" s="80">
-        <f>H$16*G$8*0.15</f>
-        <v/>
-      </c>
-      <c r="I34" s="81">
-        <f>SUM(C34:H34)</f>
-        <v/>
-      </c>
-      <c r="J34" s="75" t="inlineStr">
-        <is>
-          <t>Steal comp searches with the video.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="75" t="inlineStr">
-        <is>
-          <t>SB/Video/Comp kws-Phrase</t>
-        </is>
-      </c>
-      <c r="B35" s="74" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C35" s="80">
-        <f>C$16*B$8*0.1</f>
-        <v/>
-      </c>
-      <c r="D35" s="80">
-        <f>D$16*C$8*0.1</f>
-        <v/>
-      </c>
-      <c r="E35" s="80">
-        <f>E$16*D$8*0.1</f>
-        <v/>
-      </c>
-      <c r="F35" s="80">
-        <f>F$16*E$8*0.1</f>
-        <v/>
-      </c>
-      <c r="G35" s="80">
-        <f>G$16*F$8*0.1</f>
-        <v/>
-      </c>
-      <c r="H35" s="80">
-        <f>H$16*G$8*0.1</f>
-        <v/>
-      </c>
-      <c r="I35" s="81">
-        <f>SUM(C35:H35)</f>
-        <v/>
-      </c>
-      <c r="J35" s="75" t="inlineStr"/>
-    </row>
-    <row r="36" ht="44" customHeight="1">
-      <c r="A36" s="75" t="inlineStr">
-        <is>
-          <t>SB Brand – Product Collection (Combo-3) – ADD from M3</t>
-        </is>
-      </c>
-      <c r="B36" s="74" t="n">
-        <v>1</v>
-      </c>
-      <c r="C36" s="80">
-        <f>C$16*B$9*1.0</f>
-        <v/>
-      </c>
-      <c r="D36" s="80">
-        <f>D$16*C$9*1.0</f>
-        <v/>
-      </c>
-      <c r="E36" s="80">
-        <f>E$16*D$9*1.0</f>
-        <v/>
-      </c>
-      <c r="F36" s="80">
-        <f>F$16*E$9*1.0</f>
-        <v/>
-      </c>
-      <c r="G36" s="80">
-        <f>G$16*F$9*1.0</f>
-        <v/>
-      </c>
-      <c r="H36" s="80">
-        <f>H$16*G$9*1.0</f>
-        <v/>
-      </c>
-      <c r="I36" s="81">
-        <f>SUM(C36:H36)</f>
-        <v/>
-      </c>
-      <c r="J36" s="75" t="inlineStr">
-        <is>
-          <t>Not in your SB sheet yet. Deck: SB Brand starts M3 and sells the combo (AOV ₹450).</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="44" customHeight="1">
-      <c r="A37" s="75" t="inlineStr">
+      <c r="C50" s="80">
+        <f>B$10*B$20*1.0</f>
+        <v/>
+      </c>
+      <c r="D50" s="80">
+        <f>C$10*C$20*1.0</f>
+        <v/>
+      </c>
+      <c r="E50" s="81">
+        <f>D$10*D$20*1.0</f>
+        <v/>
+      </c>
+      <c r="F50" s="81">
+        <f>E$10*E$20*1.0</f>
+        <v/>
+      </c>
+      <c r="G50" s="82">
+        <f>F$10*F$20*1.0</f>
+        <v/>
+      </c>
+      <c r="H50" s="82">
+        <f>G$10*G$20*1.0</f>
+        <v/>
+      </c>
+      <c r="I50" s="83">
+        <f>SUM(C50:H50)</f>
+        <v/>
+      </c>
+      <c r="J50" s="97">
+        <f>ROUND(I50/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K50" s="79" t="inlineStr">
+        <is>
+          <t>Not in your SB sheet yet. Deck: SB Brand starts in M3 and sells the combo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="96" t="inlineStr">
+        <is>
+          <t>SD Retargeting   (gets 0/0/15/15/18/18% of monthly spend, M1→M6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="44" customHeight="1">
+      <c r="A52" s="79" t="inlineStr">
         <is>
           <t>SD/Remarketing/Views</t>
         </is>
       </c>
-      <c r="B37" s="74" t="inlineStr">
-        <is>
-          <t>40% (M3–4) / 35% (M5–6)</t>
-        </is>
-      </c>
-      <c r="C37" s="80">
-        <f>C$16*B$10*0.4</f>
-        <v/>
-      </c>
-      <c r="D37" s="80">
-        <f>D$16*C$10*0.4</f>
-        <v/>
-      </c>
-      <c r="E37" s="80">
-        <f>E$16*D$10*0.4</f>
-        <v/>
-      </c>
-      <c r="F37" s="80">
-        <f>F$16*E$10*0.4</f>
-        <v/>
-      </c>
-      <c r="G37" s="80">
-        <f>G$16*F$10*0.35</f>
-        <v/>
-      </c>
-      <c r="H37" s="80">
-        <f>H$16*G$10*0.35</f>
-        <v/>
-      </c>
-      <c r="I37" s="81">
-        <f>SUM(C37:H37)</f>
-        <v/>
-      </c>
-      <c r="J37" s="75" t="inlineStr">
-        <is>
-          <t>Warmest audience: saw the pack, did not buy. Deck: "retarget people who viewed".</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="44" customHeight="1">
-      <c r="A38" s="75" t="inlineStr">
+      <c r="B52" s="98" t="inlineStr">
+        <is>
+          <t>40% → 35%</t>
+        </is>
+      </c>
+      <c r="C52" s="80">
+        <f>B$10*B$21*0.4</f>
+        <v/>
+      </c>
+      <c r="D52" s="80">
+        <f>C$10*C$21*0.4</f>
+        <v/>
+      </c>
+      <c r="E52" s="81">
+        <f>D$10*D$21*0.4</f>
+        <v/>
+      </c>
+      <c r="F52" s="81">
+        <f>E$10*E$21*0.4</f>
+        <v/>
+      </c>
+      <c r="G52" s="82">
+        <f>F$10*F$21*0.35</f>
+        <v/>
+      </c>
+      <c r="H52" s="82">
+        <f>G$10*G$21*0.35</f>
+        <v/>
+      </c>
+      <c r="I52" s="83">
+        <f>SUM(C52:H52)</f>
+        <v/>
+      </c>
+      <c r="J52" s="97">
+        <f>ROUND(I52/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K52" s="79" t="inlineStr">
+        <is>
+          <t>Deck: "bring back people who viewed but did not buy" – the core SD job, so biggest SD share.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="44" customHeight="1">
+      <c r="A53" s="79" t="inlineStr">
         <is>
           <t>SD/Remarketing/Purchases</t>
         </is>
       </c>
-      <c r="B38" s="74" t="inlineStr">
-        <is>
-          <t>10% (M3–4) / 20% (M5–6)</t>
-        </is>
-      </c>
-      <c r="C38" s="80">
-        <f>C$16*B$10*0.1</f>
-        <v/>
-      </c>
-      <c r="D38" s="80">
-        <f>D$16*C$10*0.1</f>
-        <v/>
-      </c>
-      <c r="E38" s="80">
-        <f>E$16*D$10*0.1</f>
-        <v/>
-      </c>
-      <c r="F38" s="80">
-        <f>F$16*E$10*0.1</f>
-        <v/>
-      </c>
-      <c r="G38" s="80">
-        <f>G$16*F$10*0.2</f>
-        <v/>
-      </c>
-      <c r="H38" s="80">
-        <f>H$16*G$10*0.2</f>
-        <v/>
-      </c>
-      <c r="I38" s="81">
-        <f>SUM(C38:H38)</f>
-        <v/>
-      </c>
-      <c r="J38" s="75" t="inlineStr">
-        <is>
-          <t>Grows in M5–6: deck says "repeat buyers add up". One pouch = one meal, so rebuy is natural.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="75" t="inlineStr">
-        <is>
-          <t>SD/Contextual/IP (comp ASINs)</t>
-        </is>
-      </c>
-      <c r="B39" s="74" t="inlineStr">
-        <is>
-          <t>20% (M3–4) / 15% (M5–6)</t>
-        </is>
-      </c>
-      <c r="C39" s="80">
-        <f>C$16*B$10*0.2</f>
-        <v/>
-      </c>
-      <c r="D39" s="80">
-        <f>D$16*C$10*0.2</f>
-        <v/>
-      </c>
-      <c r="E39" s="80">
-        <f>E$16*D$10*0.2</f>
-        <v/>
-      </c>
-      <c r="F39" s="80">
-        <f>F$16*E$10*0.2</f>
-        <v/>
-      </c>
-      <c r="G39" s="80">
-        <f>G$16*F$10*0.15</f>
-        <v/>
-      </c>
-      <c r="H39" s="80">
-        <f>H$16*G$10*0.15</f>
-        <v/>
-      </c>
-      <c r="I39" s="81">
-        <f>SUM(C39:H39)</f>
-        <v/>
-      </c>
-      <c r="J39" s="75" t="inlineStr">
-        <is>
-          <t>Same comp ASINs as SP IP, cheaper display placement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="75" t="inlineStr">
+      <c r="B53" s="98" t="inlineStr">
+        <is>
+          <t>10% → 20%</t>
+        </is>
+      </c>
+      <c r="C53" s="80">
+        <f>B$10*B$21*0.1</f>
+        <v/>
+      </c>
+      <c r="D53" s="80">
+        <f>C$10*C$21*0.1</f>
+        <v/>
+      </c>
+      <c r="E53" s="81">
+        <f>D$10*D$21*0.1</f>
+        <v/>
+      </c>
+      <c r="F53" s="81">
+        <f>E$10*E$21*0.1</f>
+        <v/>
+      </c>
+      <c r="G53" s="82">
+        <f>F$10*F$21*0.2</f>
+        <v/>
+      </c>
+      <c r="H53" s="82">
+        <f>G$10*G$21*0.2</f>
+        <v/>
+      </c>
+      <c r="I53" s="83">
+        <f>SUM(C53:H53)</f>
+        <v/>
+      </c>
+      <c r="J53" s="97">
+        <f>ROUND(I53/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K53" s="79" t="inlineStr">
+        <is>
+          <t>Doubles in M5–6: deck says "repeat buyers add up". One pouch = one meal, so rebuy is natural.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="79" t="inlineStr">
+        <is>
+          <t>SD/Contextual/IP – comp ASINs</t>
+        </is>
+      </c>
+      <c r="B54" s="98" t="inlineStr">
+        <is>
+          <t>20% → 15%</t>
+        </is>
+      </c>
+      <c r="C54" s="80">
+        <f>B$10*B$21*0.2</f>
+        <v/>
+      </c>
+      <c r="D54" s="80">
+        <f>C$10*C$21*0.2</f>
+        <v/>
+      </c>
+      <c r="E54" s="81">
+        <f>D$10*D$21*0.2</f>
+        <v/>
+      </c>
+      <c r="F54" s="81">
+        <f>E$10*E$21*0.2</f>
+        <v/>
+      </c>
+      <c r="G54" s="82">
+        <f>F$10*F$21*0.15</f>
+        <v/>
+      </c>
+      <c r="H54" s="82">
+        <f>G$10*G$21*0.15</f>
+        <v/>
+      </c>
+      <c r="I54" s="83">
+        <f>SUM(C54:H54)</f>
+        <v/>
+      </c>
+      <c r="J54" s="97">
+        <f>ROUND(I54/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K54" s="79" t="inlineStr">
+        <is>
+          <t>Cheaper display slot on the same competitor pages as SP IP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="79" t="inlineStr">
         <is>
           <t>SD/Contextual/CT</t>
         </is>
       </c>
-      <c r="B40" s="74" t="inlineStr">
-        <is>
-          <t>15% (M3–4) / 10% (M5–6)</t>
-        </is>
-      </c>
-      <c r="C40" s="80">
-        <f>C$16*B$10*0.15</f>
-        <v/>
-      </c>
-      <c r="D40" s="80">
-        <f>D$16*C$10*0.15</f>
-        <v/>
-      </c>
-      <c r="E40" s="80">
-        <f>E$16*D$10*0.15</f>
-        <v/>
-      </c>
-      <c r="F40" s="80">
-        <f>F$16*E$10*0.15</f>
-        <v/>
-      </c>
-      <c r="G40" s="80">
-        <f>G$16*F$10*0.1</f>
-        <v/>
-      </c>
-      <c r="H40" s="80">
-        <f>H$16*G$10*0.1</f>
-        <v/>
-      </c>
-      <c r="I40" s="81">
-        <f>SUM(C40:H40)</f>
-        <v/>
-      </c>
-      <c r="J40" s="75" t="inlineStr">
-        <is>
-          <t>Category pages; cut in M5–6 (tighten, do not expand).</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="75" t="inlineStr">
+      <c r="B55" s="98" t="inlineStr">
+        <is>
+          <t>15% → 10%</t>
+        </is>
+      </c>
+      <c r="C55" s="80">
+        <f>B$10*B$21*0.15</f>
+        <v/>
+      </c>
+      <c r="D55" s="80">
+        <f>C$10*C$21*0.15</f>
+        <v/>
+      </c>
+      <c r="E55" s="81">
+        <f>D$10*D$21*0.15</f>
+        <v/>
+      </c>
+      <c r="F55" s="81">
+        <f>E$10*E$21*0.15</f>
+        <v/>
+      </c>
+      <c r="G55" s="82">
+        <f>F$10*F$21*0.1</f>
+        <v/>
+      </c>
+      <c r="H55" s="82">
+        <f>G$10*G$21*0.1</f>
+        <v/>
+      </c>
+      <c r="I55" s="83">
+        <f>SUM(C55:H55)</f>
+        <v/>
+      </c>
+      <c r="J55" s="97">
+        <f>ROUND(I55/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K55" s="79" t="inlineStr">
+        <is>
+          <t>Cut in M5–6: deck says tighten, do not expand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="30" customHeight="1">
+      <c r="A56" s="79" t="inlineStr">
         <is>
           <t>SD/Inmarketing</t>
         </is>
       </c>
-      <c r="B41" s="74" t="inlineStr">
-        <is>
-          <t>10% (M3–4) / 15% (M5–6)</t>
-        </is>
-      </c>
-      <c r="C41" s="80">
-        <f>C$16*B$10*0.1</f>
-        <v/>
-      </c>
-      <c r="D41" s="80">
-        <f>D$16*C$10*0.1</f>
-        <v/>
-      </c>
-      <c r="E41" s="80">
-        <f>E$16*D$10*0.1</f>
-        <v/>
-      </c>
-      <c r="F41" s="80">
-        <f>F$16*E$10*0.1</f>
-        <v/>
-      </c>
-      <c r="G41" s="80">
-        <f>G$16*F$10*0.15</f>
-        <v/>
-      </c>
-      <c r="H41" s="80">
-        <f>H$16*G$10*0.15</f>
-        <v/>
-      </c>
-      <c r="I41" s="81">
-        <f>SUM(C41:H41)</f>
-        <v/>
-      </c>
-      <c r="J41" s="75" t="inlineStr">
-        <is>
-          <t>New shoppers already buying spices/pastes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="75" t="inlineStr">
-        <is>
-          <t>SD/Contextual/IP (own ASINs)</t>
-        </is>
-      </c>
-      <c r="B42" s="74" t="inlineStr">
-        <is>
-          <t>5% (M3–4) / 5% (M5–6)</t>
-        </is>
-      </c>
-      <c r="C42" s="80">
-        <f>C$16*B$10*0.05</f>
-        <v/>
-      </c>
-      <c r="D42" s="80">
-        <f>D$16*C$10*0.05</f>
-        <v/>
-      </c>
-      <c r="E42" s="80">
-        <f>E$16*D$10*0.05</f>
-        <v/>
-      </c>
-      <c r="F42" s="80">
-        <f>F$16*E$10*0.05</f>
-        <v/>
-      </c>
-      <c r="G42" s="80">
-        <f>G$16*F$10*0.05</f>
-        <v/>
-      </c>
-      <c r="H42" s="80">
-        <f>H$16*G$10*0.05</f>
-        <v/>
-      </c>
-      <c r="I42" s="81">
-        <f>SUM(C42:H42)</f>
-        <v/>
-      </c>
-      <c r="J42" s="75" t="inlineStr">
+      <c r="B56" s="98" t="inlineStr">
+        <is>
+          <t>10% → 15%</t>
+        </is>
+      </c>
+      <c r="C56" s="80">
+        <f>B$10*B$21*0.1</f>
+        <v/>
+      </c>
+      <c r="D56" s="80">
+        <f>C$10*C$21*0.1</f>
+        <v/>
+      </c>
+      <c r="E56" s="81">
+        <f>D$10*D$21*0.1</f>
+        <v/>
+      </c>
+      <c r="F56" s="81">
+        <f>E$10*E$21*0.1</f>
+        <v/>
+      </c>
+      <c r="G56" s="82">
+        <f>F$10*F$21*0.15</f>
+        <v/>
+      </c>
+      <c r="H56" s="82">
+        <f>G$10*G$21*0.15</f>
+        <v/>
+      </c>
+      <c r="I56" s="83">
+        <f>SUM(C56:H56)</f>
+        <v/>
+      </c>
+      <c r="J56" s="97">
+        <f>ROUND(I56/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K56" s="79" t="inlineStr">
+        <is>
+          <t>New shoppers already buying spices / pastes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="79" t="inlineStr">
+        <is>
+          <t>SD/Contextual/IP – own ASINs</t>
+        </is>
+      </c>
+      <c r="B57" s="98" t="inlineStr">
+        <is>
+          <t>5% → 5%</t>
+        </is>
+      </c>
+      <c r="C57" s="80">
+        <f>B$10*B$21*0.05</f>
+        <v/>
+      </c>
+      <c r="D57" s="80">
+        <f>C$10*C$21*0.05</f>
+        <v/>
+      </c>
+      <c r="E57" s="81">
+        <f>D$10*D$21*0.05</f>
+        <v/>
+      </c>
+      <c r="F57" s="81">
+        <f>E$10*E$21*0.05</f>
+        <v/>
+      </c>
+      <c r="G57" s="82">
+        <f>F$10*F$21*0.05</f>
+        <v/>
+      </c>
+      <c r="H57" s="82">
+        <f>G$10*G$21*0.05</f>
+        <v/>
+      </c>
+      <c r="I57" s="83">
+        <f>SUM(C57:H57)</f>
+        <v/>
+      </c>
+      <c r="J57" s="97">
+        <f>ROUND(I57/12*0.08,0)</f>
+        <v/>
+      </c>
+      <c r="K57" s="79" t="inlineStr">
         <is>
           <t>Small defence on own pages.</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="76" t="inlineStr">
-        <is>
-          <t>Total (must match monthly spend)</t>
-        </is>
-      </c>
-      <c r="B43" s="78" t="inlineStr"/>
-      <c r="C43" s="79">
-        <f>SUM(C17:C42)</f>
-        <v/>
-      </c>
-      <c r="D43" s="79">
-        <f>SUM(D17:D42)</f>
-        <v/>
-      </c>
-      <c r="E43" s="79">
-        <f>SUM(E17:E42)</f>
-        <v/>
-      </c>
-      <c r="F43" s="79">
-        <f>SUM(F17:F42)</f>
-        <v/>
-      </c>
-      <c r="G43" s="79">
-        <f>SUM(G17:G42)</f>
-        <v/>
-      </c>
-      <c r="H43" s="79">
-        <f>SUM(H17:H42)</f>
-        <v/>
-      </c>
-      <c r="I43" s="79">
-        <f>SUM(I17:I42)</f>
-        <v/>
-      </c>
-      <c r="J43" s="78" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="69" t="inlineStr">
-        <is>
-          <t>C. Why this budget – reasons</t>
-        </is>
-      </c>
-      <c r="B46" s="70" t="n"/>
-      <c r="C46" s="70" t="n"/>
-      <c r="D46" s="70" t="n"/>
-      <c r="E46" s="70" t="n"/>
-      <c r="F46" s="70" t="n"/>
-      <c r="G46" s="70" t="n"/>
-      <c r="H46" s="70" t="n"/>
-      <c r="I46" s="70" t="n"/>
-      <c r="J46" s="71" t="n"/>
-    </row>
-    <row r="47" ht="48" customHeight="1">
-      <c r="A47" s="73" t="inlineStr">
-        <is>
-          <t>Total budget</t>
-        </is>
-      </c>
-      <c r="B47" s="75" t="inlineStr">
-        <is>
-          <t>Taken as-is from your Media Planning sheet: ₹1L (M1), ₹1L (M2), ₹2L (M3), ₹2L (M4), ₹3.33L (M5), ₹3.33L (M6) = ₹12.67L. It comes from Sales ÷ ROAS 3 (deck maths: ₹10L ÷ 3 = ₹3,33,300).</t>
-        </is>
-      </c>
-      <c r="C47" s="70" t="n"/>
-      <c r="D47" s="70" t="n"/>
-      <c r="E47" s="70" t="n"/>
-      <c r="F47" s="70" t="n"/>
-      <c r="G47" s="70" t="n"/>
-      <c r="H47" s="70" t="n"/>
-      <c r="I47" s="70" t="n"/>
-      <c r="J47" s="71" t="n"/>
-    </row>
-    <row r="48" ht="48" customHeight="1">
-      <c r="A48" s="73" t="inlineStr">
-        <is>
-          <t>Month 1–2: Get started</t>
-        </is>
-      </c>
-      <c r="B48" s="75" t="inlineStr">
-        <is>
-          <t>Deck says: fix listing, get early reviews, find best SKU. So 85% on SP (keywords + Auto + PT) to learn which keywords convert. Auto at 20% to find new keywords. No SB Brand and no SD yet – nothing to retarget and no combo push yet.</t>
-        </is>
-      </c>
-      <c r="C48" s="70" t="n"/>
-      <c r="D48" s="70" t="n"/>
-      <c r="E48" s="70" t="n"/>
-      <c r="F48" s="70" t="n"/>
-      <c r="G48" s="70" t="n"/>
-      <c r="H48" s="70" t="n"/>
-      <c r="I48" s="70" t="n"/>
-      <c r="J48" s="71" t="n"/>
-    </row>
-    <row r="49" ht="48" customHeight="1">
-      <c r="A49" s="73" t="inlineStr">
-        <is>
-          <t>Month 3–4: Grow</t>
-        </is>
-      </c>
-      <c r="B49" s="75" t="inlineStr">
-        <is>
-          <t>Deck says: spend more on what works, start brand campaigns, push combo, retarget viewers. So SB Brand (combo) starts at 10%, SD starts at 15%. Auto cut to 10% because winning search terms are moved to Exact.</t>
-        </is>
-      </c>
-      <c r="C49" s="70" t="n"/>
-      <c r="D49" s="70" t="n"/>
-      <c r="E49" s="70" t="n"/>
-      <c r="F49" s="70" t="n"/>
-      <c r="G49" s="70" t="n"/>
-      <c r="H49" s="70" t="n"/>
-      <c r="I49" s="70" t="n"/>
-      <c r="J49" s="71" t="n"/>
-    </row>
-    <row r="50" ht="48" customHeight="1">
-      <c r="A50" s="73" t="inlineStr">
-        <is>
-          <t>Month 5–6: Hit target</t>
-        </is>
-      </c>
-      <c r="B50" s="75" t="inlineStr">
-        <is>
-          <t>Deck says: tighten, do not expand; repeat buyers add up. Auto down to 8%, PT to 12%. SB Brand up to 15% (combo raises AOV). SD up to 18% with more weight on Purchase remarketing for repeat orders.</t>
-        </is>
-      </c>
-      <c r="C50" s="70" t="n"/>
-      <c r="D50" s="70" t="n"/>
-      <c r="E50" s="70" t="n"/>
-      <c r="F50" s="70" t="n"/>
-      <c r="G50" s="70" t="n"/>
-      <c r="H50" s="70" t="n"/>
-      <c r="I50" s="70" t="n"/>
-      <c r="J50" s="71" t="n"/>
-    </row>
-    <row r="51" ht="48" customHeight="1">
-      <c r="A51" s="73" t="inlineStr">
-        <is>
-          <t>Why Generic gets the most</t>
-        </is>
-      </c>
-      <c r="B51" s="75" t="inlineStr">
-        <is>
-          <t>Generic relevant searches = 4,190/month vs Brand 3,700 and Competitor 820 (your keyword sheet). New customers come from generic searches; brand searchers already know CURRYiT and are cheaper to win.</t>
-        </is>
-      </c>
-      <c r="C51" s="70" t="n"/>
-      <c r="D51" s="70" t="n"/>
-      <c r="E51" s="70" t="n"/>
-      <c r="F51" s="70" t="n"/>
-      <c r="G51" s="70" t="n"/>
-      <c r="H51" s="70" t="n"/>
-      <c r="I51" s="70" t="n"/>
-      <c r="J51" s="71" t="n"/>
-    </row>
-    <row r="52" ht="48" customHeight="1">
-      <c r="A52" s="73" t="inlineStr">
-        <is>
-          <t>Why SB Video flat 15%</t>
-        </is>
-      </c>
-      <c r="B52" s="75" t="inlineStr">
-        <is>
-          <t>Deck: "15 minute cooking video – best performing format for food". Video ads get higher CTR than static ads (benchmark ~0.9% vs 0.3–0.4%). Kept steady so the brand is always visible at top of search.</t>
-        </is>
-      </c>
-      <c r="C52" s="70" t="n"/>
-      <c r="D52" s="70" t="n"/>
-      <c r="E52" s="70" t="n"/>
-      <c r="F52" s="70" t="n"/>
-      <c r="G52" s="70" t="n"/>
-      <c r="H52" s="70" t="n"/>
-      <c r="I52" s="70" t="n"/>
-      <c r="J52" s="71" t="n"/>
-    </row>
-    <row r="53" ht="78" customHeight="1">
-      <c r="A53" s="73" t="inlineStr">
-        <is>
-          <t>Watch-outs</t>
-        </is>
-      </c>
-      <c r="B53" s="75" t="inlineStr">
-        <is>
-          <t>1) Your Media Planning assumptions table still has the Planterie text: "AOV 1000 = average of 3 plant products". CURRYiT AOV is ₹450 (combo of 3, deck). Please change it.  2) The ACOS/CTR/CPC reasons say "goes up/down gradually", but your numbers are flat (CTR 0.4%, CPC ₹12, ROAS 3 every month). Either make them change month-wise or change the text.  3) SP CT and IP campaign names in your SP sheet still say "SP/Whey Protein/…" – rename to ChettinadChicken.</t>
-        </is>
-      </c>
-      <c r="C53" s="70" t="n"/>
-      <c r="D53" s="70" t="n"/>
-      <c r="E53" s="70" t="n"/>
-      <c r="F53" s="70" t="n"/>
-      <c r="G53" s="70" t="n"/>
-      <c r="H53" s="70" t="n"/>
-      <c r="I53" s="70" t="n"/>
-      <c r="J53" s="71" t="n"/>
+    <row r="58">
+      <c r="A58" s="94" t="inlineStr">
+        <is>
+          <t>TOTAL (matches ad spend needed)</t>
+        </is>
+      </c>
+      <c r="B58" s="78" t="inlineStr"/>
+      <c r="C58" s="83">
+        <f>SUMIF($B$26:$B$57,"&lt;&gt;",C26:C57)</f>
+        <v/>
+      </c>
+      <c r="D58" s="83">
+        <f>SUMIF($B$26:$B$57,"&lt;&gt;",D26:D57)</f>
+        <v/>
+      </c>
+      <c r="E58" s="83">
+        <f>SUMIF($B$26:$B$57,"&lt;&gt;",E26:E57)</f>
+        <v/>
+      </c>
+      <c r="F58" s="83">
+        <f>SUMIF($B$26:$B$57,"&lt;&gt;",F26:F57)</f>
+        <v/>
+      </c>
+      <c r="G58" s="83">
+        <f>SUMIF($B$26:$B$57,"&lt;&gt;",G26:G57)</f>
+        <v/>
+      </c>
+      <c r="H58" s="83">
+        <f>SUMIF($B$26:$B$57,"&lt;&gt;",H26:H57)</f>
+        <v/>
+      </c>
+      <c r="I58" s="83">
+        <f>SUMIF($B$26:$B$57,"&lt;&gt;",I26:I57)</f>
+        <v/>
+      </c>
+      <c r="J58" s="87">
+        <f>SUM(J26:J57)</f>
+        <v/>
+      </c>
+      <c r="K58" s="78" t="inlineStr">
+        <is>
+          <t>Expected orders = spend ÷ CPC ₹12 × CVR 8% (deck numbers)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="70" t="inlineStr">
+        <is>
+          <t>4. Why this budget – reasons for the deck</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="46" customHeight="1">
+      <c r="A61" s="74" t="inlineStr">
+        <is>
+          <t>Why spend grows month by month</t>
+        </is>
+      </c>
+      <c r="B61" s="79" t="inlineStr">
+        <is>
+          <t>The deck gives a revenue ramp, not a flat number: ₹1.4L→₹3L, ₹3L→₹6L, ₹6L→₹10L. Spend = revenue ÷ ROAS 3, so we only spend what that month's target needs: ₹67K → ₹1L → ₹1.5L → ₹2L → ₹2.67L → ₹3.33L. Spending ₹3.33L in Month 1 with a broken listing (seller rating 2/5, 11-day delivery) would waste money.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="46" customHeight="1">
+      <c r="A62" s="74" t="inlineStr">
+        <is>
+          <t>Month 1–2: learn first</t>
+        </is>
+      </c>
+      <c r="B62" s="79" t="inlineStr">
+        <is>
+          <t>85% on SP (Exact 45 + Auto 20 + PT 20) because SP is closest to the buy. Auto + PT = 40% to find which keywords and competitor pages convert. No SB Brand (deck says M3) and no SD (no viewer pool yet).</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="46" customHeight="1">
+      <c r="A63" s="74" t="inlineStr">
+        <is>
+          <t>Month 3–4: grow what works</t>
+        </is>
+      </c>
+      <c r="B63" s="79" t="inlineStr">
+        <is>
+          <t>Winning Auto terms move to Exact, so Auto drops to 10%. SB Brand starts at 10% to push the combo (deck). SD starts at 15% because M1–2 ads have created a pool of people who viewed but did not buy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="46" customHeight="1">
+      <c r="A64" s="74" t="inlineStr">
+        <is>
+          <t>Month 5–6: tighten</t>
+        </is>
+      </c>
+      <c r="B64" s="79" t="inlineStr">
+        <is>
+          <t>Deck says tighten, do not expand. Auto 8%, PT 12%. SB Brand 15% and SD 18% – these work on people who already know CURRYiT, so they are cheaper per order and bring repeat buyers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="46" customHeight="1">
+      <c r="A65" s="74" t="inlineStr">
+        <is>
+          <t>Why Generic &gt; Brand &gt; Comp</t>
+        </is>
+      </c>
+      <c r="B65" s="79" t="inlineStr">
+        <is>
+          <t>Your keyword sheet: Generic 4,190 searches/mo, Brand 3,700, Competitor 820. Generic brings new customers. Brand shoppers already want CURRYiT, so they need less money. Competitor shoppers must be convinced to switch, so lower share.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="46" customHeight="1">
+      <c r="A66" s="74" t="inlineStr">
+        <is>
+          <t>Why SB Video is flat 15%</t>
+        </is>
+      </c>
+      <c r="B66" s="79" t="inlineStr">
+        <is>
+          <t>Deck calls it the best format for food. Video ads get ~0.9% CTR vs 0.3–0.4% for static ads (industry benchmark), so it is kept on from Month 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="46" customHeight="1">
+      <c r="A67" s="74" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="B67" s="79" t="inlineStr">
+        <is>
+          <t>Total of all campaigns = total ad spend needed every month. 6-month spend ₹11.17L for ₹33.5L revenue (ROAS 3.0). Expected ~7,444 orders.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A46:J46"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="B51:J51"/>
-    <mergeCell ref="A14:J14"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="B47:J47"/>
-    <mergeCell ref="A3:J3"/>
-    <mergeCell ref="B50:J50"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="B49:J49"/>
-    <mergeCell ref="B53:J53"/>
-    <mergeCell ref="B52:J52"/>
-    <mergeCell ref="H7:J7"/>
-    <mergeCell ref="B48:J48"/>
-    <mergeCell ref="H6:J6"/>
+  <mergeCells count="33">
+    <mergeCell ref="I16:K16"/>
+    <mergeCell ref="A24:K24"/>
+    <mergeCell ref="B65:K65"/>
+    <mergeCell ref="A49:K49"/>
+    <mergeCell ref="A51:K51"/>
+    <mergeCell ref="I18:K18"/>
+    <mergeCell ref="A60:K60"/>
+    <mergeCell ref="A36:K36"/>
+    <mergeCell ref="B64:K64"/>
+    <mergeCell ref="I21:K21"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="B63:K63"/>
+    <mergeCell ref="I5:K5"/>
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="I17:K17"/>
+    <mergeCell ref="B62:K62"/>
+    <mergeCell ref="I20:K20"/>
+    <mergeCell ref="B66:K66"/>
+    <mergeCell ref="I19:K19"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="A12:K12"/>
+    <mergeCell ref="A26:K26"/>
+    <mergeCell ref="I9:K9"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A42:K42"/>
+    <mergeCell ref="A14:K14"/>
+    <mergeCell ref="I15:K15"/>
+    <mergeCell ref="I6:K6"/>
+    <mergeCell ref="B67:K67"/>
+    <mergeCell ref="B61:K61"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A38:K38"/>
+    <mergeCell ref="I7:K7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>